<commit_message>
Deploying to gh-pages from @ mattaq31/Hash-CAD@bd86887c0f9822e81d5e1f71c8308383aa30df2c 🚀
</commit_message>
<xml_diff>
--- a/plates/cargo_plates/P3510_SSW_cnt_patterning.xlsx
+++ b/plates/cargo_plates/P3510_SSW_cnt_patterning.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10322"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10909"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/stellawang/Documents/gitrepos/Crisscross-Design/crisscross_kit/crisscross/dna_source_plates/cargo_plates/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/matt/Documents/Shih_Lab_Postdoc/research_projects/crisscross_code/crisscross_kit/crisscross/dna_source_plates/cargo_plates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B05911FD-561F-154F-B8CE-FA8DEA67AF1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A4D6517-775F-E64A-81FE-EEF5CC28B793}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-10540" yWindow="-25700" windowWidth="47420" windowHeight="21300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="51200" windowHeight="28180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="All Data" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1026" uniqueCount="757">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1041" uniqueCount="766">
   <si>
     <t>well</t>
   </si>
@@ -2293,13 +2293,40 @@
   </si>
   <si>
     <t>Obsolete well, may be contaminated, do not use</t>
+  </si>
+  <si>
+    <t>CARGO-SW066GoldNanowireAntiHandle10nt-h2-position_10</t>
+  </si>
+  <si>
+    <t>CARGO-SW066GoldNanowireAntiHandle10nt-h2-position_23</t>
+  </si>
+  <si>
+    <t>CARGO-PhosphoThio_5T-h5-position_16</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 10, Side h2, Cargo ID SW066GoldNanowireAntiHandle10nt</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 23, Side h2, Cargo ID SW066GoldNanowireAntiHandle10nt</t>
+  </si>
+  <si>
+    <t>TATTTTAAATGCCGTTCTAGCTGATAAATTGATGAACGGTAA tt ATAAAAGCAT</t>
+  </si>
+  <si>
+    <t>TAGCAAGGCCGGCGTTTTCATCGGCATTTTCAGAGCCGCCAC tt ATAAAAGCAT</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 16, Side h5, Cargo ID PhosphoThio_5T (5Ts, with 2 phosphorothioates at the end)</t>
+  </si>
+  <si>
+    <t>ACG GTG TAC ACT TTA ATC ATT GTG AAT TAA TGC GCG AAC TGA TTT* T*T</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2318,6 +2345,12 @@
     <font>
       <sz val="10"/>
       <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -2383,8 +2416,8 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4731,82 +4764,119 @@
         <v>200</v>
       </c>
     </row>
-    <row r="225" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="225" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A225" t="s">
         <v>228</v>
       </c>
-    </row>
-    <row r="226" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B225" t="s">
+        <v>757</v>
+      </c>
+      <c r="C225" s="4" t="s">
+        <v>762</v>
+      </c>
+      <c r="D225" t="s">
+        <v>760</v>
+      </c>
+      <c r="E225">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="226" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A226" t="s">
         <v>229</v>
       </c>
-    </row>
-    <row r="227" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B226" t="s">
+        <v>758</v>
+      </c>
+      <c r="C226" s="4" t="s">
+        <v>763</v>
+      </c>
+      <c r="D226" t="s">
+        <v>761</v>
+      </c>
+      <c r="E226">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="227" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A227" t="s">
         <v>230</v>
       </c>
-    </row>
-    <row r="228" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="C227" s="4"/>
+    </row>
+    <row r="228" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A228" t="s">
         <v>231</v>
       </c>
-    </row>
-    <row r="229" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B228" t="s">
+        <v>759</v>
+      </c>
+      <c r="C228" s="6" t="s">
+        <v>765</v>
+      </c>
+      <c r="D228" t="s">
+        <v>764</v>
+      </c>
+      <c r="E228">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="229" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A229" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="230" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="230" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A230" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="231" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="231" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A231" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="232" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="232" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A232" t="s">
         <v>235</v>
       </c>
     </row>
-    <row r="233" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="233" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A233" t="s">
         <v>236</v>
       </c>
     </row>
-    <row r="234" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="234" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A234" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="235" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="235" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A235" t="s">
         <v>238</v>
       </c>
     </row>
-    <row r="236" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="236" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A236" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="237" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="237" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A237" t="s">
         <v>240</v>
       </c>
     </row>
-    <row r="238" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="238" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A238" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="239" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="239" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A239" t="s">
         <v>242</v>
       </c>
     </row>
-    <row r="240" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="240" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A240" t="s">
         <v>243</v>
       </c>
@@ -6345,6 +6415,15 @@
       <c r="H11" t="s">
         <v>752</v>
       </c>
+      <c r="I11" t="s">
+        <v>757</v>
+      </c>
+      <c r="J11" t="s">
+        <v>758</v>
+      </c>
+      <c r="L11" t="s">
+        <v>759</v>
+      </c>
     </row>
     <row r="12" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
@@ -6833,19 +6912,28 @@
       <c r="B11" s="3" t="s">
         <v>736</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C11" s="5" t="s">
         <v>755</v>
       </c>
       <c r="D11" s="3" t="s">
         <v>736</v>
       </c>
-      <c r="E11" s="6" t="s">
+      <c r="E11" s="5" t="s">
         <v>755</v>
       </c>
-      <c r="G11" s="5" t="s">
-        <v>736</v>
-      </c>
-      <c r="H11" s="5" t="s">
+      <c r="G11" s="3" t="s">
+        <v>736</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>736</v>
+      </c>
+      <c r="I11" s="3" t="s">
+        <v>736</v>
+      </c>
+      <c r="J11" s="3" t="s">
+        <v>736</v>
+      </c>
+      <c r="L11" s="3" t="s">
         <v>736</v>
       </c>
     </row>

</xml_diff>